<commit_message>
Freeze validated seed 20260927 as formal Q3 and Q4
</commit_message>
<xml_diff>
--- a/outputs/q3/q3_algorithm_comparison.xlsx
+++ b/outputs/q3/q3_algorithm_comparison.xlsx
@@ -541,13 +541,13 @@
         <v>0</v>
       </c>
       <c r="J2" s="2" t="n">
-        <v>0.5619155419586445</v>
+        <v>0.5618819965228933</v>
       </c>
       <c r="K2" t="n">
         <v>0</v>
       </c>
       <c r="L2" s="2" t="n">
-        <v>18443.61177412076</v>
+        <v>18445.02405657551</v>
       </c>
     </row>
     <row r="3">
@@ -560,19 +560,19 @@
         <v>0</v>
       </c>
       <c r="C3" s="2" t="n">
-        <v>7368.139148248344</v>
+        <v>6949.848254843174</v>
       </c>
       <c r="D3" s="2" t="n">
-        <v>7368.139148248344</v>
+        <v>6949.848254843174</v>
       </c>
       <c r="E3" s="2" t="n">
-        <v>78.47952449430414</v>
+        <v>76.7409755788635</v>
       </c>
       <c r="F3" t="n">
         <v>0</v>
       </c>
       <c r="G3" s="2" t="n">
-        <v>78.47952449430414</v>
+        <v>76.7409755788635</v>
       </c>
       <c r="H3" t="n">
         <v>26</v>
@@ -591,31 +591,31 @@
         <v>0</v>
       </c>
       <c r="C4" s="2" t="n">
-        <v>7368.139148248344</v>
+        <v>6949.848254843174</v>
       </c>
       <c r="D4" s="2" t="n">
-        <v>7368.139148248344</v>
+        <v>6975.244356990602</v>
       </c>
       <c r="E4" s="2" t="n">
-        <v>78.47952449430414</v>
+        <v>76.7409755788635</v>
       </c>
       <c r="F4" s="2" t="n">
-        <v>3.599901242305765</v>
+        <v>3.348637801016601</v>
       </c>
       <c r="G4" s="2" t="n">
-        <v>82.07942573660991</v>
+        <v>80.08961337988009</v>
       </c>
       <c r="H4" t="n">
         <v>26</v>
       </c>
       <c r="I4" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="J4" s="2" t="n">
-        <v>0.5618788998126026</v>
+        <v>0.5731912702812525</v>
       </c>
       <c r="K4" s="2" t="n">
-        <v>0.4381211001873973</v>
+        <v>0.4268087297187476</v>
       </c>
       <c r="L4" t="n">
         <v>0</v>

</xml_diff>